<commit_message>
Reporte Integral de productos Financiados 14/05/2026
</commit_message>
<xml_diff>
--- a/Productos Financiados/Originacion/Version 1/Documentos/Relación de horas.xlsx
+++ b/Productos Financiados/Originacion/Version 1/Documentos/Relación de horas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Terceros\SisArrendaCredito\Productos Financiados\Originacion\Version 1\Documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6540C1D6-2D39-4B0F-9AAD-0AC9E10B836E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7243B82D-7F27-48F9-9205-6AF28D82D904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7A6E54A7-1C89-4907-9763-05848EEF796F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="24">
   <si>
     <t>Fecha</t>
   </si>
@@ -143,6 +143,12 @@
  2. Checklist Operativo
  3. Definicion de Tablas
  </t>
+  </si>
+  <si>
+    <t>Desarrollo del reporte Integral de Conceptos financiados</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -208,9 +214,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -224,6 +227,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -235,31 +241,31 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -350,15 +356,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{63582B99-8CCA-4D66-89D7-648F8ECCB686}" name="Tabla1" displayName="Tabla1" ref="A9:F25" totalsRowCount="1" headerRowDxfId="12">
-  <autoFilter ref="A9:F24" xr:uid="{63582B99-8CCA-4D66-89D7-648F8ECCB686}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{63582B99-8CCA-4D66-89D7-648F8ECCB686}" name="Tabla1" displayName="Tabla1" ref="A9:F26" totalsRowCount="1" headerRowDxfId="12">
+  <autoFilter ref="A9:F25" xr:uid="{63582B99-8CCA-4D66-89D7-648F8ECCB686}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{34329E0F-16A5-4583-9308-70D1D98D832B}" name="Fecha" dataDxfId="11" totalsRowDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{AD703B33-1671-4278-8CD6-BE420E9DC524}" name="Descripción" dataDxfId="10" totalsRowDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{A5776A45-21CC-40F2-B080-15A7417F6E0B}" name="Asistentes" dataDxfId="4" totalsRowDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{65960105-9626-4FE6-BF1D-04F8234DC8C9}" name="Hora Inicio" dataDxfId="3" totalsRowDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{E2EE5AB6-ED31-435F-A2DD-C0F565204C6D}" name="Hora Fin" dataDxfId="1" totalsRowDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{D7BAFE41-E1F9-487B-80EC-5CC4298CEFFE}" name="Horas" totalsRowFunction="sum" dataDxfId="2" totalsRowDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{34329E0F-16A5-4583-9308-70D1D98D832B}" name="Fecha" dataDxfId="11" totalsRowDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{AD703B33-1671-4278-8CD6-BE420E9DC524}" name="Descripción" dataDxfId="10" totalsRowDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{A5776A45-21CC-40F2-B080-15A7417F6E0B}" name="Asistentes" dataDxfId="9" totalsRowDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{65960105-9626-4FE6-BF1D-04F8234DC8C9}" name="Hora Inicio" dataDxfId="8" totalsRowDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{E2EE5AB6-ED31-435F-A2DD-C0F565204C6D}" name="Hora Fin" dataDxfId="7" totalsRowDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{D7BAFE41-E1F9-487B-80EC-5CC4298CEFFE}" name="Horas" totalsRowFunction="sum" dataDxfId="6" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -681,7 +687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E6A9BD7-1DE2-458E-BBC1-4A16120DB6D2}">
-  <dimension ref="A7:F25"/>
+  <dimension ref="A7:F26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="65" customWidth="1"/>
@@ -691,14 +697,14 @@
   </cols>
   <sheetData>
     <row r="7" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -730,10 +736,10 @@
       <c r="C10" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="11">
         <v>0.70833333333333337</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="11">
         <v>0.75</v>
       </c>
       <c r="F10" s="5">
@@ -750,10 +756,10 @@
       <c r="C11" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="12">
         <v>0.66666666666666663</v>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="12">
         <v>0.70833333333333304</v>
       </c>
       <c r="F11" s="5">
@@ -770,10 +776,10 @@
       <c r="C12" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="11">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E12" s="12">
+      <c r="E12" s="11">
         <v>0.58333333333333337</v>
       </c>
       <c r="F12" s="5">
@@ -786,10 +792,10 @@
         <v>11</v>
       </c>
       <c r="C13" s="4"/>
-      <c r="D13" s="13">
+      <c r="D13" s="12">
         <v>0.58333333333333337</v>
       </c>
-      <c r="E13" s="13">
+      <c r="E13" s="12">
         <v>0.83333333333333337</v>
       </c>
       <c r="F13" s="5">
@@ -804,10 +810,10 @@
         <v>12</v>
       </c>
       <c r="C14" s="4"/>
-      <c r="D14" s="13">
+      <c r="D14" s="12">
         <v>0.36805555555555558</v>
       </c>
-      <c r="E14" s="13">
+      <c r="E14" s="12">
         <v>0.63888888888888884</v>
       </c>
       <c r="F14" s="5">
@@ -820,10 +826,10 @@
         <v>13</v>
       </c>
       <c r="C15" s="4"/>
-      <c r="D15" s="13">
+      <c r="D15" s="12">
         <v>0.75</v>
       </c>
-      <c r="E15" s="13">
+      <c r="E15" s="12">
         <v>0.79166666666666663</v>
       </c>
       <c r="F15" s="5">
@@ -838,10 +844,10 @@
         <v>14</v>
       </c>
       <c r="C16" s="4"/>
-      <c r="D16" s="13">
+      <c r="D16" s="12">
         <v>0.41666666666666669</v>
       </c>
-      <c r="E16" s="13">
+      <c r="E16" s="12">
         <v>0.46875</v>
       </c>
       <c r="F16" s="5">
@@ -856,10 +862,10 @@
         <v>15</v>
       </c>
       <c r="C17" s="4"/>
-      <c r="D17" s="13">
+      <c r="D17" s="12">
         <v>0.45833333333333331</v>
       </c>
-      <c r="E17" s="13">
+      <c r="E17" s="12">
         <v>0.64236111111111116</v>
       </c>
       <c r="F17" s="5">
@@ -874,10 +880,10 @@
         <v>16</v>
       </c>
       <c r="C18" s="4"/>
-      <c r="D18" s="13">
+      <c r="D18" s="12">
         <v>0.5</v>
       </c>
-      <c r="E18" s="13">
+      <c r="E18" s="12">
         <v>0.58333333333333337</v>
       </c>
       <c r="F18" s="5">
@@ -891,13 +897,13 @@
       <c r="B19" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D19" s="13">
+      <c r="D19" s="12">
         <v>0.5</v>
       </c>
-      <c r="E19" s="13">
+      <c r="E19" s="12">
         <v>0.54166666666666663</v>
       </c>
       <c r="F19" s="5">
@@ -912,10 +918,10 @@
         <v>21</v>
       </c>
       <c r="C20" s="4"/>
-      <c r="D20" s="13">
+      <c r="D20" s="12">
         <v>0.375</v>
       </c>
-      <c r="E20" s="13">
+      <c r="E20" s="12">
         <v>0.75</v>
       </c>
       <c r="F20" s="5">
@@ -929,13 +935,13 @@
       <c r="B21" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="13">
+      <c r="D21" s="12">
         <v>0.75</v>
       </c>
-      <c r="E21" s="13">
+      <c r="E21" s="12">
         <v>0.79166666666666663</v>
       </c>
       <c r="F21" s="5">
@@ -949,11 +955,11 @@
       <c r="B22" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="10"/>
-      <c r="D22" s="13">
+      <c r="C22" s="9"/>
+      <c r="D22" s="12">
         <v>0.375</v>
       </c>
-      <c r="E22" s="13">
+      <c r="E22" s="12">
         <v>0.54166666666666663</v>
       </c>
       <c r="F22" s="5">
@@ -964,16 +970,16 @@
       <c r="A23" s="2">
         <v>46150</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D23" s="13">
+      <c r="D23" s="12">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E23" s="13">
+      <c r="E23" s="12">
         <v>0.5625</v>
       </c>
       <c r="F23" s="5">
@@ -981,21 +987,45 @@
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="2"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="5"/>
+      <c r="A24" s="2">
+        <v>46150</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="9"/>
+      <c r="D24" s="12">
+        <v>0.5625</v>
+      </c>
+      <c r="E24" s="12">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="F24" s="5">
+        <v>4</v>
+      </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="5"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="F25" s="5">
+      <c r="A25" s="2">
+        <v>46156</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" s="9"/>
+      <c r="D25" s="12">
+        <v>0.36458333333333331</v>
+      </c>
+      <c r="E25" s="12"/>
+      <c r="F25" s="5"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="5"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="F26" s="5">
         <f>SUBTOTAL(109,Tabla1[Horas])</f>
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>